<commit_message>
Formatted Excel spreadsheet for entries
</commit_message>
<xml_diff>
--- a/foresensicsspreadsheet.xlsx
+++ b/foresensicsspreadsheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ethanricks/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ethanricks/Developer/forensics-midterm/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B971344-20C5-5D4A-BCA9-1624674BE2A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25571237-E1E3-3B45-B072-4EB4A7BBC710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3260" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{ADC0C1CB-97FE-E144-9561-D3B0067A8FCF}"/>
   </bookViews>
@@ -33,6 +33,26 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>Evidence #</t>
+  </si>
+  <si>
+    <t>Type of Evidence</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Encryption Method</t>
+  </si>
+  <si>
+    <t>Decryption Method</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -402,9 +422,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56F559EB-86A4-BE49-858C-CDC4AC3D59A2}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>